<commit_message>
Resultados regenerados con nombres nuevos y test de regresion automatico
- scripts/regenerar_todo.py: regenera los 11 videos y compara viejo contra nuevo (todos identicos; 304 y 341 llevan --half-window 30)

- tests/test_regresion.py + referencia_regresion.json: regresion con un comando (--completo: desde el video)

- borrada data/processed_data/Video_068 (vigente: Video_068_hw30)

- main.py: --procesos por defecto 2 (medido en notebook de 4 nucleos)

- docs al dia (pendientes C5 y E1 hechos)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01NzBfV3TEaZuiM5M4wepfB7
</commit_message>
<xml_diff>
--- a/data/processed_data/Video_304/contracciones_Video_304.xlsx
+++ b/data/processed_data/Video_304/contracciones_Video_304.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,22 +418,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>k</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>umbral_px</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>eventos</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>falsos_control</t>
         </is>
@@ -788,172 +776,172 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>canal</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>fps</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>n_frames</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>duracion_s</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>signo</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ruido_canal_px</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>ruido_grosor_px</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>n_eventos</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>k_usado</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>k_automatico</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>hay_meseta</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>meseta_motivo</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>meseta_k_rango</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>conteo_reportable</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>cinetica_grupo_principal</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>cinetica_min_frames</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>n_eventos_cinetica</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>cinetica_motivo</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>fotogramas_sin_medida</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>fotogramas_sin_medida_pct</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>fotogramas_low_quality</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>eventos_junto_a_hueco</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>eventos_junto_al_borde</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>win_s_usado</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>win_s_automatico</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>duracion_evento_max_s</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>ventana_corta</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>conteo_por_ventana</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>conteo_estable_ventana</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>mesetas</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>motivo_no_reportable</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>ruido_borde_sup_px</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>ruido_borde_inf_px</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>cociente_ruido_bordes</t>
         </is>
@@ -981,7 +969,7 @@
         <v>0.4075667400000035</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1276465569746153</v>
+        <v>0.1276465569741939</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
B1: ventana de busqueda automatica (+-15, y +-30 si el borde se sale)
</commit_message>
<xml_diff>
--- a/data/processed_data/Video_304/contracciones_Video_304.xlsx
+++ b/data/processed_data/Video_304/contracciones_Video_304.xlsx
@@ -444,13 +444,13 @@
         <v>3</v>
       </c>
       <c r="B2" t="n">
-        <v>1.2227</v>
+        <v>1.2449</v>
       </c>
       <c r="C2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -458,13 +458,13 @@
         <v>3.3</v>
       </c>
       <c r="B3" t="n">
-        <v>1.345</v>
+        <v>1.3694</v>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -472,7 +472,7 @@
         <v>3.63</v>
       </c>
       <c r="B4" t="n">
-        <v>1.4795</v>
+        <v>1.5064</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
@@ -486,7 +486,7 @@
         <v>3.993</v>
       </c>
       <c r="B5" t="n">
-        <v>1.6274</v>
+        <v>1.657</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -500,7 +500,7 @@
         <v>4.392</v>
       </c>
       <c r="B6" t="n">
-        <v>1.79</v>
+        <v>1.8226</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
@@ -514,7 +514,7 @@
         <v>4.832</v>
       </c>
       <c r="B7" t="n">
-        <v>1.9694</v>
+        <v>2.0052</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -528,7 +528,7 @@
         <v>5.315</v>
       </c>
       <c r="B8" t="n">
-        <v>2.1662</v>
+        <v>2.2056</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
@@ -542,7 +542,7 @@
         <v>5.846</v>
       </c>
       <c r="B9" t="n">
-        <v>2.3826</v>
+        <v>2.426</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
@@ -556,7 +556,7 @@
         <v>6.431</v>
       </c>
       <c r="B10" t="n">
-        <v>2.6211</v>
+        <v>2.6687</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
@@ -570,7 +570,7 @@
         <v>7.074</v>
       </c>
       <c r="B11" t="n">
-        <v>2.8831</v>
+        <v>2.9356</v>
       </c>
       <c r="C11" t="n">
         <v>0</v>
@@ -584,7 +584,7 @@
         <v>7.781</v>
       </c>
       <c r="B12" t="n">
-        <v>3.1713</v>
+        <v>3.229</v>
       </c>
       <c r="C12" t="n">
         <v>0</v>
@@ -598,7 +598,7 @@
         <v>8.558999999999999</v>
       </c>
       <c r="B13" t="n">
-        <v>3.4884</v>
+        <v>3.5518</v>
       </c>
       <c r="C13" t="n">
         <v>0</v>
@@ -612,7 +612,7 @@
         <v>9.414999999999999</v>
       </c>
       <c r="B14" t="n">
-        <v>3.8372</v>
+        <v>3.907</v>
       </c>
       <c r="C14" t="n">
         <v>0</v>
@@ -626,7 +626,7 @@
         <v>10.357</v>
       </c>
       <c r="B15" t="n">
-        <v>4.2212</v>
+        <v>4.2979</v>
       </c>
       <c r="C15" t="n">
         <v>0</v>
@@ -640,7 +640,7 @@
         <v>11.392</v>
       </c>
       <c r="B16" t="n">
-        <v>4.643</v>
+        <v>4.7274</v>
       </c>
       <c r="C16" t="n">
         <v>0</v>
@@ -654,7 +654,7 @@
         <v>12.532</v>
       </c>
       <c r="B17" t="n">
-        <v>5.1076</v>
+        <v>5.2005</v>
       </c>
       <c r="C17" t="n">
         <v>0</v>
@@ -668,7 +668,7 @@
         <v>13.785</v>
       </c>
       <c r="B18" t="n">
-        <v>5.6183</v>
+        <v>5.7205</v>
       </c>
       <c r="C18" t="n">
         <v>0</v>
@@ -682,7 +682,7 @@
         <v>15.163</v>
       </c>
       <c r="B19" t="n">
-        <v>6.1799</v>
+        <v>6.2923</v>
       </c>
       <c r="C19" t="n">
         <v>0</v>
@@ -696,7 +696,7 @@
         <v>16.68</v>
       </c>
       <c r="B20" t="n">
-        <v>6.7982</v>
+        <v>6.9219</v>
       </c>
       <c r="C20" t="n">
         <v>0</v>
@@ -710,7 +710,7 @@
         <v>18.348</v>
       </c>
       <c r="B21" t="n">
-        <v>7.478</v>
+        <v>7.614</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
@@ -724,7 +724,7 @@
         <v>20.182</v>
       </c>
       <c r="B22" t="n">
-        <v>8.2255</v>
+        <v>8.3751</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
@@ -738,7 +738,7 @@
         <v>22.201</v>
       </c>
       <c r="B23" t="n">
-        <v>9.048400000000001</v>
+        <v>9.212999999999999</v>
       </c>
       <c r="C23" t="n">
         <v>0</v>
@@ -752,7 +752,7 @@
         <v>24.421</v>
       </c>
       <c r="B24" t="n">
-        <v>9.953200000000001</v>
+        <v>10.1342</v>
       </c>
       <c r="C24" t="n">
         <v>0</v>
@@ -966,10 +966,10 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4075667400000035</v>
+        <v>0.4149797399999968</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1276465569741939</v>
+        <v>0.1263303834691469</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -1048,13 +1048,13 @@
         </is>
       </c>
       <c r="AF2" t="n">
-        <v>0.4241718599999648</v>
+        <v>0.43054704000005</v>
       </c>
       <c r="AG2" t="n">
-        <v>0.4000054800000474</v>
+        <v>0.3995606999999906</v>
       </c>
       <c r="AH2" t="n">
-        <v>1.060415122312611</v>
+        <v>1.077551020408314</v>
       </c>
     </row>
   </sheetData>

</xml_diff>